<commit_message>
Update the PRISMA 2020 checklist against the final report
</commit_message>
<xml_diff>
--- a/Analysis/quality/prisma_checklist.xlsx
+++ b/Analysis/quality/prisma_checklist.xlsx
@@ -498,7 +498,7 @@
       </c>
       <c r="D1" s="2" t="inlineStr">
         <is>
-          <t>Where / note</t>
+          <t>Where it is reported</t>
         </is>
       </c>
     </row>
@@ -511,14 +511,14 @@
           <t>Title</t>
         </is>
       </c>
-      <c r="C2" s="3" t="inlineStr">
-        <is>
-          <t>Report</t>
+      <c r="C2" s="4" t="inlineStr">
+        <is>
+          <t>Met</t>
         </is>
       </c>
       <c r="D2" s="3" t="inlineStr">
         <is>
-          <t>To report: identify the report as a systematic review</t>
+          <t>Report cover: 'Final Project Report: a structured systematic review and evaluation framework'</t>
         </is>
       </c>
     </row>
@@ -531,14 +531,14 @@
           <t>Abstract (structured)</t>
         </is>
       </c>
-      <c r="C3" s="3" t="inlineStr">
-        <is>
-          <t>Report</t>
+      <c r="C3" s="5" t="inlineStr">
+        <is>
+          <t>Partial</t>
         </is>
       </c>
       <c r="D3" s="3" t="inlineStr">
         <is>
-          <t>To report: executive summary follows PRISMA abstract items</t>
+          <t>Executive Summary gives aim, methods, results and conclusions, but not every PRISMA abstract item</t>
         </is>
       </c>
     </row>
@@ -558,7 +558,7 @@
       </c>
       <c r="D4" s="3" t="inlineStr">
         <is>
-          <t>Proposal s.1; Project Context s.2</t>
+          <t>Report Section 1 (the business problem and the opportunity)</t>
         </is>
       </c>
     </row>
@@ -578,7 +578,7 @@
       </c>
       <c r="D5" s="3" t="inlineStr">
         <is>
-          <t>RQ1-RQ5 (proposal)</t>
+          <t>Report Section 1.2 (research questions RQ1 to RQ5)</t>
         </is>
       </c>
     </row>
@@ -598,7 +598,7 @@
       </c>
       <c r="D6" s="3" t="inlineStr">
         <is>
-          <t>IC1-IC5, E1-E7; Amendment 3 (redesign focus), dated</t>
+          <t>Report Section 3.2; Literature Review Evidence, sheet 'Read me and methods' (criteria IC1 to IC5, exclusion codes E1 to E7, dated redesign amendment)</t>
         </is>
       </c>
     </row>
@@ -618,7 +618,7 @@
       </c>
       <c r="D7" s="3" t="inlineStr">
         <is>
-          <t>Team evidence log + OpenAlex update search, dates recorded</t>
+          <t>Report Section 3.2 and Figure 1: team evidence log and an OpenAlex update search on 17 October 2026</t>
         </is>
       </c>
     </row>
@@ -638,7 +638,7 @@
       </c>
       <c r="D8" s="3" t="inlineStr">
         <is>
-          <t>Update search strings fully recorded; original team searches not recorded</t>
+          <t>Update-search strings recorded in full in the code repository (screening/search/search_log.csv); the original team searches were not recorded (Report Section 3.2)</t>
         </is>
       </c>
     </row>
@@ -658,7 +658,7 @@
       </c>
       <c r="D9" s="3" t="inlineStr">
         <is>
-          <t>Two independent AI-assisted screeners (separate model runs, B blinded to A) with a human adjudicator for every disagreement; AI assistance disclosed</t>
+          <t>Report Section 3.2: two independent AI-assisted screening runs, the second blinded to the first, with a team member settling every disagreement; AI use disclosed in Section 3.6</t>
         </is>
       </c>
     </row>
@@ -678,7 +678,7 @@
       </c>
       <c r="D10" s="3" t="inlineStr">
         <is>
-          <t>Written extraction protocol; full or light extraction stated</t>
+          <t>Report Section 3.2: written extraction protocol recording each finding with its location in the source (protocol in the code repository)</t>
         </is>
       </c>
     </row>
@@ -698,7 +698,7 @@
       </c>
       <c r="D11" s="3" t="inlineStr">
         <is>
-          <t>Protocol key list (design, sample, findings with locations, dimensions)</t>
+          <t>Literature Review Evidence, sheet 'Study details' (design, sample, findings with locations, notes on each criterion)</t>
         </is>
       </c>
     </row>
@@ -718,7 +718,7 @@
       </c>
       <c r="D12" s="3" t="inlineStr">
         <is>
-          <t>5-item checklist adapted from MMAT 2018 / CASP</t>
+          <t>Report Section 3.2: five-item checklist adapted from MMAT 2018; Literature Review Evidence, sheet 'Quality appraisal'</t>
         </is>
       </c>
     </row>
@@ -738,7 +738,7 @@
       </c>
       <c r="D13" s="3" t="inlineStr">
         <is>
-          <t>Narrative / qualitative synthesis; no pooled effect sizes</t>
+          <t>Framework synthesis of mixed evidence; no pooled effect sizes (Report Section 3.5)</t>
         </is>
       </c>
     </row>
@@ -758,7 +758,7 @@
       </c>
       <c r="D14" s="3" t="inlineStr">
         <is>
-          <t>Structured framework synthesis, D2 protocol and calibration rules C1-C4</t>
+          <t>Report Section 3.4: framework synthesis with written calibration rules; D2 Evaluation Framework, sheet 'Read me'</t>
         </is>
       </c>
     </row>
@@ -778,7 +778,7 @@
       </c>
       <c r="D15" s="3" t="inlineStr">
         <is>
-          <t>Venue credibility check and sensitivity analysis; no formal publication-bias test</t>
+          <t>Venue credibility check and sensitivity analysis (Report Section 6); no formal publication-bias test</t>
         </is>
       </c>
     </row>
@@ -798,7 +798,7 @@
       </c>
       <c r="D16" s="3" t="inlineStr">
         <is>
-          <t>Simplified GRADE-CERQual (High / Medium / Low per finding)</t>
+          <t>Report Section 3.4: CERQual-informed confidence rule (High, Medium or Low for every rating)</t>
         </is>
       </c>
     </row>
@@ -818,7 +818,7 @@
       </c>
       <c r="D17" s="3" t="inlineStr">
         <is>
-          <t>prisma_counts_combined.csv; diagram to draw in report</t>
+          <t>Report Figure 1 (PRISMA flow diagram); Literature Review Evidence, sheet 'PRISMA'</t>
         </is>
       </c>
     </row>
@@ -838,7 +838,7 @@
       </c>
       <c r="D18" s="3" t="inlineStr">
         <is>
-          <t>Included studies sheet (design, setting, sample, discipline)</t>
+          <t>Literature Review Evidence, sheets 'Included studies' and 'Study details'; Report Section 4.1</t>
         </is>
       </c>
     </row>
@@ -858,7 +858,7 @@
       </c>
       <c r="D19" s="3" t="inlineStr">
         <is>
-          <t>Quality score per study</t>
+          <t>Quality score for every study (Literature Review Evidence, sheet 'Quality appraisal'); summary in Report Section 4.1</t>
         </is>
       </c>
     </row>
@@ -878,7 +878,7 @@
       </c>
       <c r="D20" s="3" t="inlineStr">
         <is>
-          <t>Key findings with source locations</t>
+          <t>Literature Review Evidence, sheet 'Study details' (findings with their location in each source)</t>
         </is>
       </c>
     </row>
@@ -898,7 +898,7 @@
       </c>
       <c r="D21" s="3" t="inlineStr">
         <is>
-          <t>D2 cells with [L]/[D]/[I] evidence</t>
+          <t>Report Section 4.3; D2 Evaluation Framework, sheets 'Rating Grid' and 'Cell Evidence'</t>
         </is>
       </c>
     </row>
@@ -918,7 +918,7 @@
       </c>
       <c r="D22" s="3" t="inlineStr">
         <is>
-          <t>Low-confidence venues flagged; sensitivity check shows no cell depends on them</t>
+          <t>Low-confidence venues flagged; sensitivity checks without them and without the two most-cited studies change no rating (Report Section 6)</t>
         </is>
       </c>
     </row>
@@ -938,7 +938,7 @@
       </c>
       <c r="D23" s="3" t="inlineStr">
         <is>
-          <t>Confidence per D2 cell; evidence status per D3 recommendation</t>
+          <t>Report Section 4.3 (confidence for every D2 rating) and Section 5 (evidence status for every D3 recommendation)</t>
         </is>
       </c>
     </row>
@@ -951,14 +951,14 @@
           <t>Discussion and limitations</t>
         </is>
       </c>
-      <c r="C24" s="3" t="inlineStr">
-        <is>
-          <t>Report</t>
+      <c r="C24" s="4" t="inlineStr">
+        <is>
+          <t>Met</t>
         </is>
       </c>
       <c r="D24" s="3" t="inlineStr">
         <is>
-          <t>To report: limits listed in D2/D3 and summary</t>
+          <t>Report Section 6 (limits of the evidence) and Section 9 (conclusion)</t>
         </is>
       </c>
     </row>
@@ -978,7 +978,7 @@
       </c>
       <c r="D25" s="3" t="inlineStr">
         <is>
-          <t>Protocols written and dated; review not registered (e.g. PROSPERO/OSF)</t>
+          <t>Protocols written and dated in the code repository; the review was not registered (for example on PROSPERO or OSF)</t>
         </is>
       </c>
     </row>
@@ -991,14 +991,14 @@
           <t>Support / funding</t>
         </is>
       </c>
-      <c r="C26" s="3" t="inlineStr">
-        <is>
-          <t>Report</t>
+      <c r="C26" s="4" t="inlineStr">
+        <is>
+          <t>Met</t>
         </is>
       </c>
       <c r="D26" s="3" t="inlineStr">
         <is>
-          <t>To report</t>
+          <t>Report Section 8.2: no external funding; tool costs from the project budget</t>
         </is>
       </c>
     </row>
@@ -1011,14 +1011,14 @@
           <t>Competing interests</t>
         </is>
       </c>
-      <c r="C27" s="3" t="inlineStr">
-        <is>
-          <t>Report</t>
+      <c r="C27" s="4" t="inlineStr">
+        <is>
+          <t>Met</t>
         </is>
       </c>
       <c r="D27" s="3" t="inlineStr">
         <is>
-          <t>To report</t>
+          <t>Report Section 8.2: the team declares no competing interests</t>
         </is>
       </c>
     </row>
@@ -1038,7 +1038,7 @@
       </c>
       <c r="D28" s="3" t="inlineStr">
         <is>
-          <t>All scripts and outputs in Analysis/ with READMEs</t>
+          <t>Report Appendix A: code repository and supplementary documents (links)</t>
         </is>
       </c>
     </row>
@@ -1053,7 +1053,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B5"/>
+  <dimension ref="A1:B4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -1079,13 +1079,13 @@
         </is>
       </c>
       <c r="B2" s="3" t="n">
-        <v>17</v>
+        <v>21</v>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="3" t="inlineStr">
-        <is>
-          <t>Report</t>
+      <c r="A3" s="5" t="inlineStr">
+        <is>
+          <t>Partial</t>
         </is>
       </c>
       <c r="B3" s="3" t="n">
@@ -1093,22 +1093,12 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="5" t="inlineStr">
-        <is>
-          <t>Partial</t>
+      <c r="A4" s="3" t="inlineStr">
+        <is>
+          <t>Not applicable</t>
         </is>
       </c>
       <c r="B4" s="3" t="n">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="3" t="inlineStr">
-        <is>
-          <t>Not applicable</t>
-        </is>
-      </c>
-      <c r="B5" s="3" t="n">
         <v>1</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Update PRISMA checklist figure references
</commit_message>
<xml_diff>
--- a/Analysis/quality/prisma_checklist.xlsx
+++ b/Analysis/quality/prisma_checklist.xlsx
@@ -618,7 +618,7 @@
       </c>
       <c r="D7" s="3" t="inlineStr">
         <is>
-          <t>Report Section 3.2 and Figure 1: team evidence log and an OpenAlex update search on 17 October 2026</t>
+          <t>Report Section 3.2 and Figure 2: team evidence log and an OpenAlex update search on 17 October 2026</t>
         </is>
       </c>
     </row>
@@ -818,7 +818,7 @@
       </c>
       <c r="D17" s="3" t="inlineStr">
         <is>
-          <t>Report Figure 1 (PRISMA flow diagram); Literature Review Evidence, sheet 'PRISMA'</t>
+          <t>Report Figure 2 (PRISMA flow diagram); Literature Review Evidence, sheet 'PRISMA'</t>
         </is>
       </c>
     </row>

</xml_diff>